<commit_message>
fix: cambios en documentación, código, layout de archivos
</commit_message>
<xml_diff>
--- a/res/importancias_variables.xlsx
+++ b/res/importancias_variables.xlsx
@@ -1003,7 +1003,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>V3_Zócalo (con madera, zinc o fibrocemento)</t>
+          <t>V3_Zócalo</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>V15_Otra fuente o sin electricidad</t>
+          <t>V15_Otro o no tiene</t>
         </is>
       </c>
       <c r="B93" t="n">

</xml_diff>